<commit_message>
Take the Barclaycard payee from "Beschreibung"
The Barclaycard export changed: "Beschreibung" now holds the name of
the payee, the details of the transaction moved to "Details", which the
parser already uses for the info field. For card payments, type
"Belastung", the payee is now taken from "Beschreibung" as it is,
without removing spaces. Other types keep an empty payee.

The fixtures follow the current layout: the former "Beschreibung"
texts moved to "Details", "Beschreibung" holds synthetic payee names,
and a "Gutschrift" row covers a type without payee.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UDkWYL8TWAXyjmV37vrvty
</commit_message>
<xml_diff>
--- a/internal/pkg/batchconvert/testfiles/input/mixed/Umsaetze.xlsx
+++ b/internal/pkg/batchconvert/testfiles/input/mixed/Umsaetze.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr showObjects="all"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId3" state="visible"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
+  <calcPr iterateCount="100" iterateDelta="0.001" refMode="A1"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
   <si>
     <t xml:space="preserve">Transaktionsansicht</t>
   </si>
@@ -251,49 +251,88 @@
   </si>
   <si>
     <t xml:space="preserve">Detail6</t>
+  </si>
+  <si>
+    <t>Kiosk Am Markt</t>
+  </si>
+  <si>
+    <t>KIOSK AM MARKT     BERLIN     DE</t>
+  </si>
+  <si>
+    <t>PayPal Europe</t>
+  </si>
+  <si>
+    <t>XYZ  Rotterdam</t>
+  </si>
+  <si>
+    <t>Abc</t>
+  </si>
+  <si>
+    <t>DB Fernverkehr AG</t>
+  </si>
+  <si>
+    <t>Bank Ort</t>
+  </si>
+  <si>
+    <t>DB Bahn</t>
+  </si>
+  <si>
+    <t>98765432109876543210993</t>
+  </si>
+  <si>
+    <t>08.09.2020</t>
+  </si>
+  <si>
+    <t>20,00 €</t>
+  </si>
+  <si>
+    <t>Gutschrift</t>
+  </si>
+  <si>
+    <t>Erstattung DB Bahn</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0"/>
   </numFmts>
   <fonts count="6">
     <font>
+      <name val="Calibri"/>
+      <charset val="1"/>
+      <family val="0"/>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+      <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <charset val="1"/>
+      <family val="0"/>
       <sz val="16"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <charset val="1"/>
+      <family val="0"/>
       <sz val="10"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -311,14 +350,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left style="thin"/>
       <right style="thin"/>
       <top style="thin"/>
@@ -328,8 +367,8 @@
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+      <alignment horizontal="general" vertical="bottom"/>
+      <protection hidden="false" locked="true"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
@@ -353,24 +392,24 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+      <alignment horizontal="general" vertical="bottom"/>
+      <protection hidden="false" locked="true"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+      <alignment horizontal="general" vertical="bottom"/>
+      <protection hidden="false" locked="true"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+      <alignment horizontal="general" vertical="bottom"/>
+      <protection hidden="false" locked="true"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="false" locked="true"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+      <alignment horizontal="left" vertical="center"/>
+      <protection hidden="false" locked="true"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -487,14 +526,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial" pitchFamily="0"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial" pitchFamily="0"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -547,40 +586,42 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+  <sheetPr>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O20"/>
-  <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="12.8"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="27.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="13.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="38.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="10.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="19.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="5.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="23.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="14.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="21.64"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="11.63"/>
+    <col customWidth="true" max="1" min="1" style="1" width="23.56"/>
+    <col customWidth="true" max="2" min="2" style="1" width="27.42"/>
+    <col customWidth="true" max="4" min="3" style="1" width="13.94"/>
+    <col customWidth="true" max="5" min="5" style="1" width="38.96"/>
+    <col customWidth="true" max="7" min="6" style="1" width="10.09"/>
+    <col customWidth="true" max="8" min="8" style="1" width="16.83"/>
+    <col customWidth="true" max="9" min="9" style="1" width="14.89"/>
+    <col customWidth="true" max="10" min="10" style="1" width="19.71"/>
+    <col customWidth="true" max="11" min="11" style="1" width="5.28"/>
+    <col customWidth="true" max="12" min="12" style="1" width="23.56"/>
+    <col customWidth="true" max="13" min="13" style="1" width="14.89"/>
+    <col customWidth="true" max="14" min="14" style="1" width="21.64"/>
+    <col customWidth="true" max="15" min="15" style="1" width="11.63"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" ht="13.8"/>
+    <row r="2" ht="19.7">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" ht="13.8"/>
+    <row r="4" ht="13.8">
       <c r="A4" s="3" t="s">
         <v>1</v>
       </c>
@@ -588,7 +629,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" ht="13.8">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -596,7 +637,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" ht="13.8">
       <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
@@ -604,7 +645,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" ht="13.8">
       <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
@@ -612,7 +653,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" ht="13.8">
       <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
@@ -620,7 +661,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" ht="13.8">
       <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
@@ -628,7 +669,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" ht="13.8">
       <c r="A10" s="3" t="s">
         <v>13</v>
       </c>
@@ -636,7 +677,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" ht="13.8">
       <c r="A11" s="3" t="s">
         <v>15</v>
       </c>
@@ -644,8 +685,8 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" ht="13.8"/>
+    <row r="13" ht="12.8">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -692,7 +733,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" ht="13.8">
       <c r="A14" s="4" t="s">
         <v>30</v>
       </c>
@@ -703,7 +744,7 @@
         <v>32</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>33</v>
+        <v>77</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>34</v>
@@ -730,10 +771,10 @@
         <v>38</v>
       </c>
       <c r="O14" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="15" ht="12.8">
       <c r="A15" s="4" t="s">
         <v>42</v>
       </c>
@@ -747,7 +788,7 @@
         <v>44</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>45</v>
+        <v>79</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>34</v>
@@ -777,10 +818,10 @@
         <v>38</v>
       </c>
       <c r="O15" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" ht="12.8">
       <c r="A16" s="4" t="s">
         <v>49</v>
       </c>
@@ -794,7 +835,7 @@
         <v>52</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>53</v>
+        <v>80</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>34</v>
@@ -822,10 +863,10 @@
         <v>38</v>
       </c>
       <c r="O16" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" ht="12.8">
       <c r="A17" s="4" t="s">
         <v>55</v>
       </c>
@@ -839,7 +880,7 @@
         <v>58</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>34</v>
@@ -869,10 +910,10 @@
         <v>38</v>
       </c>
       <c r="O17" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" ht="12.8">
       <c r="A18" s="4" t="s">
         <v>61</v>
       </c>
@@ -886,7 +927,7 @@
         <v>62</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>34</v>
@@ -916,10 +957,10 @@
         <v>38</v>
       </c>
       <c r="O18" s="4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" ht="12.8">
       <c r="A19" s="4" t="s">
         <v>65</v>
       </c>
@@ -933,7 +974,7 @@
         <v>67</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>34</v>
@@ -963,10 +1004,10 @@
         <v>38</v>
       </c>
       <c r="O19" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="20" ht="12.8">
       <c r="A20" s="4" t="s">
         <v>71</v>
       </c>
@@ -980,7 +1021,7 @@
         <v>74</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>34</v>
@@ -1010,16 +1051,60 @@
         <v>38</v>
       </c>
       <c r="O20" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="M21" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="N21" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="O21" s="1" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <printOptions gridLinesSet="true"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup cellComments="none" copies="1" fitToHeight="1" fitToWidth="1" horizontalDpi="300" orientation="portrait" pageOrder="downThenOver" paperSize="9" scale="100" verticalDpi="300"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Keep the formatting of the Barclaycard fixtures
Saving the fixtures with excelize rewrote the whole workbook: the added
"Gutschrift" row got the default style without borders, and
Umsaetze_shortrows.xlsx had no formatting at all already before.

Rebuild both from the formatted Umsaetze.xlsx of main by editing only
the cell values in sheet1.xml and sharedStrings.xml. The new rows use
the bordered style of the other data rows; all other parts of the
workbook stay unchanged. The content read by the parser is the same as
before.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UDkWYL8TWAXyjmV37vrvty
</commit_message>
<xml_diff>
--- a/internal/pkg/batchconvert/testfiles/input/mixed/Umsaetze.xlsx
+++ b/internal/pkg/batchconvert/testfiles/input/mixed/Umsaetze.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr showObjects="all"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId3" state="visible"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr iterateCount="100" iterateDelta="0.001" refMode="A1"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="90">
   <si>
     <t xml:space="preserve">Transaktionsansicht</t>
   </si>
@@ -253,86 +253,86 @@
     <t xml:space="preserve">Detail6</t>
   </si>
   <si>
-    <t>Kiosk Am Markt</t>
-  </si>
-  <si>
-    <t>KIOSK AM MARKT     BERLIN     DE</t>
-  </si>
-  <si>
-    <t>PayPal Europe</t>
-  </si>
-  <si>
-    <t>XYZ  Rotterdam</t>
-  </si>
-  <si>
-    <t>Abc</t>
-  </si>
-  <si>
-    <t>DB Fernverkehr AG</t>
-  </si>
-  <si>
-    <t>Bank Ort</t>
-  </si>
-  <si>
-    <t>DB Bahn</t>
-  </si>
-  <si>
-    <t>98765432109876543210993</t>
-  </si>
-  <si>
-    <t>08.09.2020</t>
-  </si>
-  <si>
-    <t>20,00 €</t>
-  </si>
-  <si>
-    <t>Gutschrift</t>
-  </si>
-  <si>
-    <t>Erstattung DB Bahn</t>
+    <t xml:space="preserve">Kiosk Am Markt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KIOSK AM MARKT     BERLIN     DE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PayPal Europe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XYZ  Rotterdam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DB Fernverkehr AG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bank Ort</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DB Bahn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">98765432109876543210993</t>
+  </si>
+  <si>
+    <t xml:space="preserve">08.09.2020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20,00 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gutschrift</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erstattung DB Bahn</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0"/>
   </numFmts>
   <fonts count="6">
     <font>
+      <sz val="11"/>
       <name val="Calibri"/>
+      <family val="0"/>
       <charset val="1"/>
-      <family val="0"/>
-      <sz val="11"/>
     </font>
     <font>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-      <sz val="10"/>
     </font>
     <font>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-      <sz val="10"/>
     </font>
     <font>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-      <sz val="10"/>
     </font>
     <font>
+      <sz val="16"/>
       <name val="Calibri"/>
+      <family val="0"/>
       <charset val="1"/>
-      <family val="0"/>
-      <sz val="16"/>
     </font>
     <font>
+      <sz val="10"/>
       <name val="Calibri"/>
+      <family val="0"/>
       <charset val="1"/>
-      <family val="0"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -350,14 +350,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left style="thin"/>
       <right style="thin"/>
       <top style="thin"/>
@@ -367,8 +367,8 @@
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom"/>
-      <protection hidden="false" locked="true"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
@@ -392,24 +392,24 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom"/>
-      <protection hidden="false" locked="true"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom"/>
-      <protection hidden="false" locked="true"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom"/>
-      <protection hidden="false" locked="true"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="false" locked="true"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center"/>
-      <protection hidden="false" locked="true"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -526,14 +526,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0"/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0"/>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -586,42 +586,40 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr>
-    <pageSetUpPr/>
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O20"/>
-  <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="12.8"/>
+  <dimension ref="A1:O21"/>
+  <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col customWidth="true" max="1" min="1" style="1" width="23.56"/>
-    <col customWidth="true" max="2" min="2" style="1" width="27.42"/>
-    <col customWidth="true" max="4" min="3" style="1" width="13.94"/>
-    <col customWidth="true" max="5" min="5" style="1" width="38.96"/>
-    <col customWidth="true" max="7" min="6" style="1" width="10.09"/>
-    <col customWidth="true" max="8" min="8" style="1" width="16.83"/>
-    <col customWidth="true" max="9" min="9" style="1" width="14.89"/>
-    <col customWidth="true" max="10" min="10" style="1" width="19.71"/>
-    <col customWidth="true" max="11" min="11" style="1" width="5.28"/>
-    <col customWidth="true" max="12" min="12" style="1" width="23.56"/>
-    <col customWidth="true" max="13" min="13" style="1" width="14.89"/>
-    <col customWidth="true" max="14" min="14" style="1" width="21.64"/>
-    <col customWidth="true" max="15" min="15" style="1" width="11.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="27.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="13.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="38.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="10.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="19.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="5.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="23.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="14.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="21.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="11.63"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.8"/>
-    <row r="2" ht="19.7">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" ht="13.8"/>
-    <row r="4" ht="13.8">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>1</v>
       </c>
@@ -629,7 +627,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" ht="13.8">
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -637,7 +635,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" ht="13.8">
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
@@ -645,7 +643,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" ht="13.8">
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
@@ -653,7 +651,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" ht="13.8">
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
@@ -661,7 +659,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" ht="13.8">
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
@@ -669,7 +667,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" ht="13.8">
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
         <v>13</v>
       </c>
@@ -677,7 +675,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" ht="13.8">
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
         <v>15</v>
       </c>
@@ -685,8 +683,8 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" ht="13.8"/>
-    <row r="13" ht="12.8">
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
         <v>17</v>
       </c>
@@ -733,7 +731,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" ht="13.8">
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
         <v>30</v>
       </c>
@@ -774,7 +772,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="15" ht="12.8">
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
         <v>42</v>
       </c>
@@ -821,7 +819,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" ht="12.8">
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
         <v>49</v>
       </c>
@@ -866,7 +864,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="17" ht="12.8">
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
         <v>55</v>
       </c>
@@ -913,7 +911,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="18" ht="12.8">
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
         <v>61</v>
       </c>
@@ -960,7 +958,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="19" ht="12.8">
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
         <v>65</v>
       </c>
@@ -1007,7 +1005,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="20" ht="12.8">
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
         <v>71</v>
       </c>
@@ -1054,57 +1052,60 @@
         <v>75</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="1" t="s">
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D21" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="E21" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="F21" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="G21" s="1" t="s">
+      <c r="G21" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H21" s="1" t="s">
+      <c r="H21" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="I21" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="J21" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="K21" s="1" t="s">
+      <c r="J21" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="K21" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="L21" s="1" t="s">
+      <c r="L21" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="M21" s="1" t="s">
+      <c r="M21" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="N21" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="O21" s="1" t="s">
+      <c r="N21" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O21" s="4" t="s">
         <v>89</v>
       </c>
     </row>
   </sheetData>
-  <printOptions gridLinesSet="true"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup cellComments="none" copies="1" fitToHeight="1" fitToWidth="1" horizontalDpi="300" orientation="portrait" pageOrder="downThenOver" paperSize="9" scale="100" verticalDpi="300"/>
-  <headerFooter/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>